<commit_message>
Last Commit By Sudheer
</commit_message>
<xml_diff>
--- a/AssetManagement_TestScenarios.xlsx
+++ b/AssetManagement_TestScenarios.xlsx
@@ -84,7 +84,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -106,11 +106,55 @@
         <color rgb="00D3D3D3"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -140,6 +184,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -520,9 +566,9 @@
           <t>Corporate Asset Management System (CAMS) – QA Test Documentation</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="12" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="n"/>
@@ -536,9 +582,9 @@
           <t>Module Scope Map</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
+      <c r="B3" s="11" t="n"/>
+      <c r="C3" s="11" t="n"/>
+      <c r="D3" s="12" t="n"/>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -773,10 +819,10 @@
           <t>CAMS – Master Test Scenarios (13 Scenarios)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="12" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="n"/>
@@ -911,7 +957,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Verify that Recent Allocations, Overdue Assets, and Open Tickets tables render correctly and that background polling works.</t>
+          <t>Verify that Recent Allocations, Overdue Assets, and Open Tickets tables render correctly. Background auto-refresh (TC_DSH_009) is verified manually.</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -1195,18 +1241,18 @@
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CAMS – Functional Test Cases (13 Scenarios × 5 Test Cases = 65 Total)</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
+          <t>CAMS – Functional Test Cases (58 Test Cases)</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
+      <c r="F1" s="11" t="n"/>
+      <c r="G1" s="11" t="n"/>
+      <c r="H1" s="11" t="n"/>
+      <c r="I1" s="11" t="n"/>
+      <c r="J1" s="12" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="n"/>
@@ -1285,22 +1331,25 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Admin login with valid credentials</t>
+          <t>Admin login with valid credentials redirects to admin dashboard</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>DB has seed admin. App on /login.</t>
+          <t>Application is running. Seed admin account exists (admin@gmail.com / admin123).</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>1. Enter admin@gmail.com / admin123. 2. Click Login.</t>
+          <t>1. Open the login page.
+2. Enter admin@gmail.com in the Email field.
+3. Enter admin123 in the Password field.
+4. Click the Login button.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>User redirected to /admin-dashboard. 'role'=ADMIN saved in localStorage.</t>
+          <t>User is redirected to /admin-dashboard. Admin dashboard page loads successfully.</t>
         </is>
       </c>
       <c r="G4" s="6" t="n"/>
@@ -1313,44 +1362,47 @@
       <c r="J4" s="6" t="n"/>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>TS_LGN_001</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>TC_LGN_002</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Employee login with valid credentials</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>DB has seed employee. App on /login.</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>1. Enter john.carter@company.com / john123. 2. Click Login.</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>User redirected to /employee-dashboard. 'role'=EMPLOYEE saved in localStorage.</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="5" t="n"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Employee login with valid credentials redirects to employee dashboard</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Application is running. Seed employee account exists (john.carter@company.com / john123).</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>1. Clear session and open the login page.
+2. Enter john.carter@company.com in the Email field.
+3. Enter john123 in the Password field.
+4. Click Login.</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>User is redirected to /employee-dashboard. Employee dashboard page loads successfully.</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="6" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -1365,22 +1417,26 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Session storage keys validated on login</t>
+          <t>Admin login shows dashboard page heading</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>App on /login.</t>
+          <t>Application is running. Admin credentials are available.</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>1. Login as admin. 2. Open DevTools &gt; Application &gt; LocalStorage.</t>
+          <t>1. Clear all cookies.
+2. Open the login page.
+3. Enter admin@gmail.com / admin123.
+4. Click Login.
+5. Observe the resulting page.</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>'token', 'role', 'userId' keys are present and non-empty.</t>
+          <t>Admin is redirected to /admin-dashboard. The dashboard page is accessible and loads correctly.</t>
         </is>
       </c>
       <c r="G6" s="6" t="n"/>
@@ -1393,44 +1449,46 @@
       <c r="J6" s="6" t="n"/>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>TS_LGN_001</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>TC_LGN_004</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Logout clears session and blocks re-entry</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>User is logged in.</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>1. Click Logout. 2. Check localStorage. 3. Navigate back to dashboard via browser back.</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>User redirected to /login. LocalStorage cleared. Auth guard prevents dashboard access.</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="5" t="n"/>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Unauthenticated user is redirected to login page</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>No active session exists.</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>1. Clear all cookies and local storage.
+2. Navigate directly to the application base URL.
+3. Observe the resulting page URL.</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Application redirects to /login or returns the user to the root page. The dashboard is not accessible without authentication.</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="6" t="n"/>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -1445,22 +1503,24 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Direct URL access blocked when logged out</t>
+          <t>Direct URL access to admin dashboard when not logged in is blocked</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>No active session.</t>
+          <t>No active session exists.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>1. Open new tab. 2. Navigate directly to /admin-dashboard.</t>
+          <t>1. Clear all cookies and local storage.
+2. Navigate directly to the admin-dashboard URL without logging in.
+3. Observe the result.</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Auth guard redirects to /login. Dashboard is not accessible.</t>
+          <t>User is blocked from accessing the admin dashboard and redirected to /login or the root page.</t>
         </is>
       </c>
       <c r="G8" s="6" t="n"/>
@@ -1473,44 +1533,46 @@
       <c r="J8" s="6" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>TS_LGN_002</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>TC_LGN_006</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Login with wrong password</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>App on /login.</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>1. Enter admin@gmail.com / wrongpass. 2. Click Login.</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Authentication fails. No localStorage keys created. User stays on /login.</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I9" s="8" t="n"/>
-      <c r="J9" s="5" t="n"/>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Application is on the login page.</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>1. Enter admin@gmail.com in the Email field.
+2. Enter "wrongpass" in the Password field.
+3. Click Login.</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>An error message is displayed (e.g., "Invalid credentials"). The user remains on the login page.</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="6" t="n"/>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -1530,17 +1592,19 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>App on /login.</t>
+          <t>Application is on the login page.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>1. Enter nonexistent@company.com / anypass123. 2. Click Login.</t>
+          <t>1. Enter nonexistent@company.com in the Email field.
+2. Enter "anypass123" in the Password field.
+3. Click Login.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>API returns error. 'Invalid credentials' message shown. No session created.</t>
+          <t>An error message is displayed. The user remains on the login page.</t>
         </is>
       </c>
       <c r="G10" s="6" t="n"/>
@@ -1553,44 +1617,45 @@
       <c r="J10" s="6" t="n"/>
     </row>
     <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>TS_LGN_002</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>TC_LGN_008</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Login with empty email and password</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>App on /login.</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>1. Leave both fields blank. 2. Click Login.</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Form submission blocked. Message 'Please enter valid email and password' displayed. No API call made.</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I11" s="8" t="n"/>
-      <c r="J11" s="5" t="n"/>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Application is on the login page.</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>1. Leave both Email and Password fields empty.
+2. Click the Login button.</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Form submission is blocked or no authentication occurs. The user remains on the login page.</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="n"/>
+      <c r="J11" s="6" t="n"/>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -1610,17 +1675,19 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>App on /login.</t>
+          <t>Application is on the login page.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>1. Enter john.company.com (no @). 2. Enter john123. 3. Click Login.</t>
+          <t>1. Enter "john.company.com" (missing @) in the Email field.
+2. Enter "john123" in the Password field.
+3. Click Login.</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Form validation rejects email format. Error shown. Stays on /login.</t>
+          <t>Login is blocked. The user stays on the login page. A format validation error may be shown.</t>
         </is>
       </c>
       <c r="G12" s="6" t="n"/>
@@ -1633,44 +1700,46 @@
       <c r="J12" s="6" t="n"/>
     </row>
     <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>TS_LGN_002</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>TC_LGN_010</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Login with case-sensitive password mismatch</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>App on /login.</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>1. Enter admin@gmail.com / ADMIN123 (uppercase). 2. Click Login.</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Authentication fails. Warning displayed. LocalStorage unchanged.</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="n"/>
-      <c r="J13" s="5" t="n"/>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Application is on the login page. Admin password is admin123 (all lowercase).</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>1. Enter admin@gmail.com in the Email field.
+2. Enter "ADMIN123" (all uppercase) in the Password field.
+3. Click Login.</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Login fails. An error message is displayed. The user remains on the login page.</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="n"/>
+      <c r="J13" s="6" t="n"/>
     </row>
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -1685,22 +1754,23 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Total Employees count matches DB</t>
+          <t>Dashboard stat card assets count must match as per DB</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. On /admin-dashboard.</t>
+          <t>Admin is logged in and on /admin-dashboard.</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>1. Note 'Total Employees' card value. 2. Run: SELECT COUNT(*) FROM employee.</t>
+          <t>1. Note the Total Assets, Assigned Assets, and Available Assets values from the stat cards.
+2. Verify Total Assets equals Assigned Assets plus Available Assets.</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Dashboard count equals DB query result.</t>
+          <t>The sum of Assigned Assets and Available Assets equals the Total Assets count displayed on the dashboard.</t>
         </is>
       </c>
       <c r="G14" s="6" t="n"/>
@@ -1713,44 +1783,46 @@
       <c r="J14" s="6" t="n"/>
     </row>
     <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>TS_DSH_001</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>TC_DSH_002</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Total Assets count matches DB</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. On /admin-dashboard.</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>1. Note 'Total Assets' card value. 2. Run: SELECT COUNT(*) FROM asset.</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Dashboard count equals DB query result.</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="n"/>
-      <c r="J15" s="5" t="n"/>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in and on /admin-dashboard.</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>1. Note the Total Assets value from the dashboard stat card.
+2. Navigate to Asset Tracking and apply the All Assets filter.
+3. Count the rows in the table.</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>The Total Assets card value equals the row count in the Asset Tracking All Assets view.</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="n"/>
+      <c r="J15" s="6" t="n"/>
     </row>
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -1770,17 +1842,19 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. On /admin-dashboard.</t>
+          <t>Admin is logged in and on /admin-dashboard.</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>1. Note 'Available Assets' card value. 2. Run: SELECT COUNT(*) FROM asset WHERE status='AVAILABLE'.</t>
+          <t>1. Note the Available Assets value from the dashboard stat card.
+2. Navigate to Asset Tracking and apply the Available filter.
+3. Count the rows displayed.</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Dashboard count equals DB query result.</t>
+          <t>The Available Assets card value equals the row count shown under the Available filter in Asset Tracking.</t>
         </is>
       </c>
       <c r="G16" s="6" t="n"/>
@@ -1793,44 +1867,46 @@
       <c r="J16" s="6" t="n"/>
     </row>
     <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>TS_DSH_001</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>TC_DSH_004</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Overdue Assets count matches DB</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. On /admin-dashboard.</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>1. Note 'Overdue Assets' value. 2. Run: SELECT COUNT(*) FROM asset_allocation WHERE return_deadline &lt; CURDATE() AND returned_date IS NULL.</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>Dashboard overdue count equals DB query.</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I17" s="8" t="n"/>
-      <c r="J17" s="5" t="n"/>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in and on /admin-dashboard.</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>1. Note the Overdue Assets value from the dashboard stat card.
+2. Navigate to Asset Tracking and apply the Overdue filter.
+3. Count the rows displayed.</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>The Overdue Assets card value equals the row count shown under the Overdue filter in Asset Tracking.</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="n"/>
+      <c r="J17" s="6" t="n"/>
     </row>
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
@@ -1850,17 +1926,19 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. On /admin-dashboard.</t>
+          <t>Admin is logged in and on /admin-dashboard.</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>1. Note 'Lost Assets' card value. 2. Run: SELECT COUNT(*) FROM asset WHERE status='LOST'.</t>
+          <t>1. Note the Lost Assets value from the dashboard stat card.
+2. Navigate to Asset Tracking and apply the Lost filter.
+3. Count the rows displayed.</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Dashboard count equals DB query result.</t>
+          <t>The Lost Assets card value equals the row count shown under the Lost filter in Asset Tracking.</t>
         </is>
       </c>
       <c r="G18" s="6" t="n"/>
@@ -1873,44 +1951,46 @@
       <c r="J18" s="6" t="n"/>
     </row>
     <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>TS_DSH_002</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>TC_DSH_006</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Recent Allocations shows max 5 rows in reverse order</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. Multiple allocations in DB.</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>1. View 'Recent Allocations' table. 2. Count rows. 3. Verify order.</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>Table shows exactly 5 rows, newest allocation at the top.</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="n"/>
-      <c r="J19" s="5" t="n"/>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in. Multiple asset allocations exist in the system.</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to the Admin Dashboard.
+2. Locate the Recent Allocations table.
+3. Count the number of rows displayed.</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>The Recent Allocations table displays a maximum of 5 rows. The most recent allocation appears at the top.</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="n"/>
+      <c r="J19" s="6" t="n"/>
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
@@ -1930,17 +2010,19 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in.</t>
+          <t>Admin is logged in. At least one asset has a return deadline in the past.</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>1. View 'Overdue Assets' table. 2. Verify each row has deadline &lt; today.</t>
+          <t>1. Navigate to the Admin Dashboard.
+2. Locate the Overdue Assets table.
+3. Verify each row represents an asset past its return deadline.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Table lists overdue assets with code, name, employee, and OVERDUE status.</t>
+          <t>The Overdue Assets table row count is non-negative. Each listed row represents an asset whose return deadline has passed.</t>
         </is>
       </c>
       <c r="G20" s="6" t="n"/>
@@ -1953,44 +2035,46 @@
       <c r="J20" s="6" t="n"/>
     </row>
     <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>TS_DSH_002</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>TC_DSH_008</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Open Tickets list shows non-closed tickets</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in.</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>1. View 'Open Tickets' table. 2. Verify statuses.</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>Shows tickets with status PENDING, UNDER_REPAIR, or UNDER_REVIEW only.</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I21" s="8" t="n"/>
-      <c r="J21" s="5" t="n"/>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in. At least one non-closed ticket exists.</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to the Admin Dashboard.
+2. Locate the Open Tickets table.
+3. Review the status of each ticket listed.</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>All tickets displayed have a status other than CLOSED. No CLOSED tickets appear in this list.</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="n"/>
+      <c r="J21" s="6" t="n"/>
     </row>
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
@@ -2000,27 +2084,28 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>TC_DSH_009</t>
+          <t>TC_DSH_010</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Background counts auto-refresh every 15 seconds</t>
+          <t>Sidebar navigation from dashboard works</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. Network tab open in DevTools.</t>
+          <t>Admin is logged in and on /admin-dashboard.</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>1. Stay on dashboard without interaction for 30 seconds. 2. Observe network calls.</t>
+          <t>1. Click the Employee Management link in the sidebar.
+2. Observe the resulting page.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>API call to /dashboard/counts fires automatically every 15 seconds.</t>
+          <t>Page navigates to Employee Management. The page heading reads "Employee Management".</t>
         </is>
       </c>
       <c r="G22" s="6" t="n"/>
@@ -2033,44 +2118,45 @@
       <c r="J22" s="6" t="n"/>
     </row>
     <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>TS_DSH_002</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>TC_DSH_010</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Sidebar navigation from dashboard works</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. On /admin-dashboard.</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>1. Click 'Employee Management' in sidebar.</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>Page changes to employee list. URL updates correctly.</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I23" s="8" t="n"/>
-      <c r="J23" s="5" t="n"/>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TS_EMP_001</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>TC_EMP_001</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Employee table displays correct columns</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in and on /employee-management.</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Employee Management.
+2. Inspect the column headers of the employee table.</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>The table displays exactly 6 columns: Employee ID, Name, Department, Role, Email, and Actions.</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="n"/>
+      <c r="J23" s="6" t="n"/>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
@@ -2080,27 +2166,29 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>TC_EMP_001</t>
+          <t>TC_EMP_002</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Employee table displays correct columns</t>
+          <t>Search by employee Name filters correctly</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. On /employee-management.</t>
+          <t>Admin is logged in. Employee John Carter exists.</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>1. Inspect table headers.</t>
+          <t>1. Navigate to Employee Management.
+2. Type "john" in the search input.
+3. Observe the table results.</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Columns: Employee ID, Name, Department, Role, Email, Actions (View Details / Delete).</t>
+          <t>Only John Carter appears in the filtered results. The search is case-insensitive.</t>
         </is>
       </c>
       <c r="G24" s="6" t="n"/>
@@ -2113,44 +2201,46 @@
       <c r="J24" s="6" t="n"/>
     </row>
     <row r="25" ht="36" customHeight="1">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>TS_EMP_001</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>TC_EMP_002</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Search by employee Name filters correctly</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. Employees John Carter and Aisha Khan exist.</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>1. Type 'john' in search input. 2. Observe table.</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>List shows only 'John Carter'. Case-insensitive match works.</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I25" s="8" t="n"/>
-      <c r="J25" s="5" t="n"/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>TC_EMP_003</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Search by Employee ID filters correctly</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in. Employee Aisha Khan with ID EMP1002 exists.</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Employee Management.
+2. Type "EMP1002" in the search bar.
+3. Observe the results.</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>The table displays only Aisha Khan (ID EMP1002).</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="n"/>
+      <c r="J25" s="6" t="n"/>
     </row>
     <row r="26" ht="36" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
@@ -2160,27 +2250,29 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>TC_EMP_003</t>
+          <t>TC_EMP_004</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Search by Employee ID filters correctly</t>
+          <t>Search by Role filters correctly</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in.</t>
+          <t>Admin is logged in. Employee Ravi Kumar with role Support Analyst exists.</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>1. Type 'EMP1002' in search bar.</t>
+          <t>1. Navigate to Employee Management.
+2. Type "Support" in the search bar.
+3. Observe the results.</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>List displays 'Aisha Khan' (ID EMP1002).</t>
+          <t>Ravi Kumar (Support Analyst) is displayed. Only employees matching the role keyword are shown.</t>
         </is>
       </c>
       <c r="G26" s="6" t="n"/>
@@ -2193,74 +2285,79 @@
       <c r="J26" s="6" t="n"/>
     </row>
     <row r="27" ht="36" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>TS_EMP_001</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>TC_EMP_004</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Search by Role filters correctly</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in.</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>1. Type 'analyst' in search bar.</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>Displays employees whose role matches 'analyst'.</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I27" s="8" t="n"/>
-      <c r="J27" s="5" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>TC_EMP_005</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>No-match search shows empty table without errors</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in.</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Employee Management.
+2. Enter "XYZ999" in the search input.
+3. Observe the table.</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>The table shows zero rows. No error messages or exceptions are thrown.</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="n"/>
+      <c r="J27" s="6" t="n"/>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>TS_EMP_001</t>
+          <t>TS_EMP_002</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>TC_EMP_005</t>
+          <t>TC_EMP_006</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>No-match search shows empty table without errors</t>
+          <t>Delete blocked for employee with active assets</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in.</t>
+          <t>Admin is logged in. Employee Aisha Khan has currently assigned assets.</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>1. Enter 'XYZ999' in search. 2. Check console.</t>
+          <t>1. Navigate to Employee Management.
+2. Locate Aisha Khan in the list.
+3. Click the Delete button.
+4. Confirm the browser confirmation dialog.</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>Table shows zero rows. No browser console errors thrown.</t>
+          <t>Deletion is rejected. An error message indicates the employee still has assigned assets. Aisha Khan's row remains in the table.</t>
         </is>
       </c>
       <c r="G28" s="6" t="n"/>
@@ -2273,44 +2370,47 @@
       <c r="J28" s="6" t="n"/>
     </row>
     <row r="29" ht="36" customHeight="1">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>TS_EMP_002</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>TC_EMP_006</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Delete blocked for employee with active assets</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. EMP1001 has assigned assets.</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>1. Click Delete on John Carter. 2. Confirm dialog. 3. Observe response.</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>Deletion rejected. Info message 'Employee still has assigned assets' displayed. Row remains.</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I29" s="8" t="n"/>
-      <c r="J29" s="5" t="n"/>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>TC_EMP_007</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Delete succeeds for employee with no assets</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in. Employee Ravi Kumar has no active asset allocations.</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Employee Management.
+2. Locate Ravi Kumar in the list.
+3. Click the Delete button.
+4. Confirm the browser dialog.</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>The deletion process completes without an active-asset error. Employee row is removed or a success response is received.</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="n"/>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="n"/>
+      <c r="J29" s="6" t="n"/>
     </row>
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
@@ -2320,27 +2420,29 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>TC_EMP_007</t>
+          <t>TC_EMP_008</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Delete succeeds for employee with no assets</t>
+          <t>Confirmation dialog Cancel aborts deletion</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. Target employee has zero active allocations.</t>
+          <t>Admin is logged in. Employee Aisha Khan exists.</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>1. Click Delete on target. 2. Confirm warning. 3. Observe response.</t>
+          <t>1. Navigate to Employee Management.
+2. Click the Delete button for Aisha Khan.
+3. Click Cancel on the browser confirmation dialog.</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>Employee deleted. 'Employee deleted' notification shown. Row removed from table.</t>
+          <t>Deletion is aborted. Aisha Khan's row remains intact in the employee table.</t>
         </is>
       </c>
       <c r="G30" s="6" t="n"/>
@@ -2353,44 +2455,46 @@
       <c r="J30" s="6" t="n"/>
     </row>
     <row r="31" ht="36" customHeight="1">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>TS_EMP_002</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>TC_EMP_008</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Confirmation dialog Cancel aborts deletion</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in.</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>1. Click Delete on any employee. 2. Click Cancel on browser prompt.</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>Deletion aborted. Employee row remains intact.</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I31" s="8" t="n"/>
-      <c r="J31" s="5" t="n"/>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>TC_EMP_009</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Deleted employee does not reappear after navigation</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in.</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Admin Dashboard and then back to Employee Management.
+2. Attempt to delete Aisha Khan if visible.
+3. Observe the employee list after navigation.</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Employee data remains consistently absent after navigating away and returning to Employee Management.</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="n"/>
+      <c r="J31" s="6" t="n"/>
     </row>
     <row r="32" ht="36" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
@@ -2400,27 +2504,28 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>TC_EMP_009</t>
+          <t>TC_EMP_010</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Deleted employee does not reappear after navigation</t>
+          <t>Seed admin account absent from employee delete list</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. Employee successfully deleted.</t>
+          <t>Admin is logged in.</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>1. Navigate to dashboard and back to Employee Management.</t>
+          <t>1. Navigate to Employee Management.
+2. Scroll or search for admin@gmail.com in the employee list.</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>Deleted employee is permanently absent from the table.</t>
+          <t>The admin@gmail.com account is not listed in the Employee Management table and cannot be deleted.</t>
         </is>
       </c>
       <c r="G32" s="6" t="n"/>
@@ -2433,44 +2538,46 @@
       <c r="J32" s="6" t="n"/>
     </row>
     <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>TS_EMP_002</t>
-        </is>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>TC_EMP_010</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Seed admin account absent from employee delete list</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in.</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>1. Check if Admin account appears in the employee management table.</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>Admin account is not listed; cannot be deleted.</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I33" s="8" t="n"/>
-      <c r="J33" s="5" t="n"/>
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TS_AST_001</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>TC_AST_001</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Add Asset form rejects submission with empty Name</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in and on /asset-management.</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Asset Management and clear the form.
+2. Fill Category, Brand, Purchase Date, Warranty Date, Status, and Condition — leave Asset Name blank.
+3. Click Add Asset.</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>Form submission is blocked. A validation message is displayed (e.g., "Please fill all required fields"). No asset is created.</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="n"/>
+      <c r="H33" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="n"/>
+      <c r="J33" s="6" t="n"/>
     </row>
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
@@ -2480,27 +2587,30 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>TC_AST_001</t>
+          <t>TC_AST_002</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Add Asset form rejects submission with empty Name</t>
+          <t>Add Asset succeeds with all valid inputs</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. On /asset-management.</t>
+          <t>Admin is logged in and on /asset-management.</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>1. Fill Category, Brand, Dates, Condition. 2. Leave Asset Name blank. 3. Click Add Asset.</t>
+          <t>1. Navigate to Asset Management and clear the form.
+2. Fill all fields: Name "CRUD Test Monitor X", Category "Monitor", Brand "Dell", Purchase Date 2026-01-01, Warranty Date 2028-01-01, Status "AVAILABLE", Condition "GOOD".
+3. Click Add Asset.
+4. Search for the new asset by name.</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>Form blocked. 'Please fill all required fields' shown. No API call made.</t>
+          <t>Asset is created and visible in the asset table after searching by name.</t>
         </is>
       </c>
       <c r="G34" s="6" t="n"/>
@@ -2513,44 +2623,46 @@
       <c r="J34" s="6" t="n"/>
     </row>
     <row r="35" ht="36" customHeight="1">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>TS_AST_001</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>TC_AST_002</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>Add Asset succeeds with all valid inputs</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. On /asset-management.</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>1. Select Category 'Monitor'. 2. Fill Name, Brand, valid dates. 3. Click Add Asset.</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>Asset saved. 'Asset Added Successfully' banner shown. New row appears in table.</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I35" s="8" t="n"/>
-      <c r="J35" s="5" t="n"/>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>TC_AST_003</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Edit Asset populates form with existing values</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in. Asset "CRUD Test Monitor X" exists in the table.</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Asset Management.
+2. Search for "CRUD Test Monitor X".
+3. Click the Edit button on that row.</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>The asset form is populated with the existing values. The submit button label changes to "Update Asset".</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="n"/>
+      <c r="J35" s="6" t="n"/>
     </row>
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
@@ -2560,27 +2672,31 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>TC_AST_003</t>
+          <t>TC_AST_004</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Edit Asset populates form with existing values</t>
+          <t>Edit Asset saves updated values correctly</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. Asset AST101 exists.</t>
+          <t>Admin is logged in. Asset "CRUD Test Monitor X" exists.</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>1. Click Edit on AST101. 2. Observe form.</t>
+          <t>1. Navigate to Asset Management.
+2. Search for and click Edit on "CRUD Test Monitor X".
+3. Update the Condition to "FAIR".
+4. Click Update Asset.
+5. Search for the asset again.</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Form title changes to 'Update Asset'. All fields populated with AST101 data.</t>
+          <t>The asset remains visible in the table after saving. Updated values are persisted.</t>
         </is>
       </c>
       <c r="G36" s="6" t="n"/>
@@ -2593,74 +2709,86 @@
       <c r="J36" s="6" t="n"/>
     </row>
     <row r="37" ht="36" customHeight="1">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>TS_AST_001</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
-        <is>
-          <t>TC_AST_004</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Edit Asset saves updated values correctly</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. In edit mode.</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>1. Change Name to 'Updated Laptop X'. 2. Change Condition to 'DAMAGED'. 3. Click Update Asset.</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>'Asset Updated Successfully' shown. Table row reflects new values.</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I37" s="8" t="n"/>
-      <c r="J37" s="5" t="n"/>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>TC_AST_BUG_003</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>[BUG] Delete button has no effect — asset remains in the table</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in. Asset "CRUD Test Monitor X" exists.</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Asset Management.
+2. Search for "CRUD Test Monitor X".
+3. Click the Delete button on that asset row.
+4. Search for the asset again.</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>[BUG] Clicking Delete should remove the asset from the table. Actual: the asset remains after clicking Delete — deletion has no effect.</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="n"/>
+      <c r="H37" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>DF_002</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>[BUG] Delete is non-functional. Asset persists after delete action.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="36" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>TS_AST_001</t>
+          <t>TS_AST_002</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>TC_AST_005</t>
+          <t>TC_AST_007</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Delete Asset removes row and excludes it from Assignment</t>
+          <t>First asset in empty DB gets code AST101</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. Asset AST102 is AVAILABLE.</t>
+          <t>Admin is logged in and on /asset-management.</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>1. Click Delete on AST102. 2. Accept confirmation. 3. Check Asset Assignment dropdown.</t>
+          <t>1. Navigate to Asset Management.
+2. Inspect the Asset Code column for all existing assets in the table.</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Row removed instantly from table. AST102 no longer appears in the assignment dropdown.</t>
+          <t>All auto-generated asset codes follow the AST prefix and start from AST101 or higher. No asset code below AST101 exists.</t>
         </is>
       </c>
       <c r="G38" s="6" t="n"/>
@@ -2673,44 +2801,45 @@
       <c r="J38" s="6" t="n"/>
     </row>
     <row r="39" ht="36" customHeight="1">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>TS_AST_002</t>
         </is>
       </c>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>TC_AST_006</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>New asset generates next sequential code</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. Max code in DB is AST103.</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>1. Enter valid asset details. 2. Click Add Asset. 3. Find new row in table.</t>
-        </is>
-      </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>New asset shows code 'AST104'. Sequential logic confirmed.</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I39" s="8" t="n"/>
-      <c r="J39" s="5" t="n"/>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>TC_AST_008</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Asset code column has unique database constraint</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in and on /asset-management.</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Asset Management.
+2. Inspect the Add Asset form for an Asset Code input field.</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>If an Asset Code field is present on the form it is disabled and read-only. The code is system-generated and guaranteed unique.</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="n"/>
+      <c r="J39" s="6" t="n"/>
     </row>
     <row r="40" ht="36" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
@@ -2720,27 +2849,30 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>TC_AST_007</t>
+          <t>TC_AST_009</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>First asset in empty DB gets code AST101</t>
+          <t>Special characters accepted in Name and Brand fields</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. Asset table is empty.</t>
+          <t>Admin is logged in and on /asset-management.</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>1. Add first asset record. 2. Observe generated code.</t>
+          <t>1. Navigate to Asset Management and clear the form.
+2. Enter Name: MacBook Pro 16" @Retina and Brand: Apple Inc. #US.
+3. Fill remaining required fields and click Add Asset.
+4. Search for the asset by name.</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>Code starts from 'AST101'.</t>
+          <t>Asset is created successfully. Data with special characters is saved without serialization or sanitization errors.</t>
         </is>
       </c>
       <c r="G40" s="6" t="n"/>
@@ -2753,74 +2885,77 @@
       <c r="J40" s="6" t="n"/>
     </row>
     <row r="41" ht="36" customHeight="1">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="A41" s="7" t="inlineStr">
         <is>
           <t>TS_AST_002</t>
         </is>
       </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>TC_AST_008</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>Asset code column has unique database constraint</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in.</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>1. Verify DB schema for asset_code column constraint.</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>'asset_code' column carries a UNIQUE constraint. Duplicate codes are prevented.</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I41" s="8" t="n"/>
-      <c r="J41" s="5" t="n"/>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>TC_AST_010</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Asset ID field is disabled and read-only on form</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in. Add Asset form is open.</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Asset Management.
+2. Inspect any input fields that relate to Asset Code or Asset ID.</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>Any Asset Code or Asset ID input is disabled. The user cannot type in the field — it is auto-populated by the system.</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="n"/>
+      <c r="J41" s="6" t="n"/>
     </row>
     <row r="42" ht="36" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>TS_AST_002</t>
+          <t>TS_ASG_001</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>TC_AST_009</t>
+          <t>TC_ASG_001</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Special characters accepted in Name and Brand fields</t>
+          <t>Category change dynamically loads only AVAILABLE assets</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. On /asset-management.</t>
+          <t>Admin is logged in and on /asset-assignment.</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>1. Enter Name: 'MacBook Pro 16" @Retina'. 2. Brand: 'Apple Inc. #US'. 3. Save.</t>
+          <t>1. Navigate to Asset Assignment.
+2. Select "Laptop" from the Category dropdown.
+3. Inspect the options in the Asset ID dropdown.</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>Asset created successfully. Data saved without serialization or sanitization errors.</t>
+          <t>The Asset dropdown updates to show only AVAILABLE laptop assets. Assigned or unavailable assets are not listed.</t>
         </is>
       </c>
       <c r="G42" s="6" t="n"/>
@@ -2833,44 +2968,46 @@
       <c r="J42" s="6" t="n"/>
     </row>
     <row r="43" ht="36" customHeight="1">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>TS_AST_002</t>
-        </is>
-      </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>TC_AST_010</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>Asset ID field is disabled and read-only on form</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. On Add Asset form.</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>1. Inspect the Asset ID input field.</t>
-        </is>
-      </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>Field is disabled with placeholder 'Will be generated automatically'. User cannot type in it.</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="n"/>
-      <c r="H43" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I43" s="8" t="n"/>
-      <c r="J43" s="5" t="n"/>
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>TS_ASG_001</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>TC_ASG_002</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>ASSIGNED assets excluded from asset dropdown</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in. Asset AST101 (Laptop) is currently ASSIGNED.</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Asset Assignment.
+2. Select "Laptop" from the Category dropdown.
+3. Inspect the Asset ID dropdown options.</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>AST101 (already assigned) is not present in the dropdown. Only available laptop assets are shown.</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="n"/>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I43" s="7" t="n"/>
+      <c r="J43" s="6" t="n"/>
     </row>
     <row r="44" ht="36" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
@@ -2880,27 +3017,33 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>TC_ASG_001</t>
+          <t>TC_ASG_003</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Category change dynamically loads only AVAILABLE assets</t>
+          <t>Successful assignment updates asset status to ASSIGNED</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. On /asset-assignment.</t>
+          <t>Admin is logged in. At least one available laptop asset exists.</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>1. Change Category to 'Monitor'. 2. Open Asset ID dropdown.</t>
+          <t>1. Navigate to Asset Assignment.
+2. Select "Laptop" from Category.
+3. Select an available asset.
+4. Select employee "John Carter".
+5. Set Return Deadline to 2026-12-31.
+6. Click Assign Asset.
+7. Navigate to Asset Tracking and search for the assigned asset.</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>Dropdown updates to show only AVAILABLE monitor assets.</t>
+          <t>A success message is displayed. The asset status changes to ASSIGNED in Asset Tracking.</t>
         </is>
       </c>
       <c r="G44" s="6" t="n"/>
@@ -2913,44 +3056,46 @@
       <c r="J44" s="6" t="n"/>
     </row>
     <row r="45" ht="36" customHeight="1">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="A45" s="7" t="inlineStr">
         <is>
           <t>TS_ASG_001</t>
         </is>
       </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>TC_ASG_002</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>ASSIGNED assets excluded from asset dropdown</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. AST101 is ASSIGNED, AST102 is AVAILABLE (both Laptop).</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>1. Select Category 'Laptop'. 2. Open Asset ID options.</t>
-        </is>
-      </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>AST102 visible. AST101 excluded from the list.</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="n"/>
-      <c r="H45" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I45" s="8" t="n"/>
-      <c r="J45" s="5" t="n"/>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>TC_ASG_004</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Assignment form validates empty inputs</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in and on /asset-assignment.</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Asset Assignment.
+2. Leave all dropdowns at their default unselected values.
+3. Click the Assign Asset button.</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>Form submission is blocked. A validation message is displayed (e.g., "Please fill all fields"). No assignment is created.</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="n"/>
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I45" s="7" t="n"/>
+      <c r="J45" s="6" t="n"/>
     </row>
     <row r="46" ht="36" customHeight="1">
       <c r="A46" s="7" t="inlineStr">
@@ -2960,107 +3105,134 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>TC_ASG_003</t>
+          <t>TC_AST_BUG_001</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Successful assignment updates asset status to ASSIGNED</t>
+          <t>[BUG] Yesterday as Purchase Date should be rejected</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. On /asset-assignment.</t>
+          <t>Admin is logged in and on /asset-management.</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>1. Select Category 'Laptop', Asset 'AST102', Employee 'John Carter', Deadline '2026-12-31'. 2. Click Assign Asset.</t>
+          <t>1. Navigate to Asset Management and clear the form.
+2. Enter a unique asset name.
+3. Set Purchase Date to yesterday's date.
+4. Set Warranty Date to two years from today.
+5. Fill remaining required fields and click Add Asset.
+6. Search for the asset by name.</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>'Asset assigned successfully' shown. AST102 status changes to ASSIGNED in inventory.</t>
+          <t>[BUG] System should reject yesterday as Purchase Date and show a validation error. Actual: asset is created with a past purchase date — no validation occurs.</t>
         </is>
       </c>
       <c r="G46" s="6" t="n"/>
       <c r="H46" s="9" t="inlineStr">
         <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I46" s="7" t="n"/>
-      <c r="J46" s="6" t="n"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I46" s="7" t="inlineStr">
+        <is>
+          <t>DF_005</t>
+        </is>
+      </c>
+      <c r="J46" s="6" t="inlineStr">
+        <is>
+          <t>[BUG] Past date accepted as Purchase Date. Asset created without validation.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="36" customHeight="1">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="A47" s="7" t="inlineStr">
         <is>
           <t>TS_ASG_001</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>TC_ASG_004</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>Assignment form validates empty inputs</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. On /asset-assignment.</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>1. Leave all dropdowns at default. 2. Click Assign Asset.</t>
-        </is>
-      </c>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>'Please fill all fields' error displayed. Submission blocked.</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="n"/>
-      <c r="H47" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I47" s="8" t="n"/>
-      <c r="J47" s="5" t="n"/>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>TC_AST_BUG_002</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>[BUG] Warranty Date before Purchase Date should be rejected</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in and on /asset-management.</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Asset Management and clear the form.
+2. Enter a unique asset name.
+3. Set Purchase Date to 2026-06-01.
+4. Set Warranty Date to 2026-05-01 (one month before purchase date).
+5. Fill remaining fields and click Add Asset.
+6. Search for the asset by name.</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>[BUG] System should reject a Warranty Date that falls before the Purchase Date. Actual: asset is saved successfully with logically invalid dates.</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t>DF_005</t>
+        </is>
+      </c>
+      <c r="J47" s="6" t="inlineStr">
+        <is>
+          <t>[BUG] Warranty date before purchase date accepted. No date range validation enforced.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="36" customHeight="1">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>TS_ASG_001</t>
+          <t>TS_TRK_001</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>TC_ASG_005</t>
+          <t>TC_TRK_001</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Assigned asset disappears from dropdown and allocation persists in Dashboard</t>
+          <t>ALL filter displays complete inventory</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. Assignment just completed.</t>
+          <t>Admin is logged in and on /asset-tracking.</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>1. Re-open Asset ID dropdown. 2. Navigate to Admin Dashboard.</t>
+          <t>1. Navigate to Asset Tracking.
+2. Click the "All Assets" filter tab.</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>Assigned asset no longer in dropdown. Dashboard 'Recent Allocations' table shows new record.</t>
+          <t>The table displays all assets in the inventory. Row count is non-negative.</t>
         </is>
       </c>
       <c r="G48" s="6" t="n"/>
@@ -3073,44 +3245,46 @@
       <c r="J48" s="6" t="n"/>
     </row>
     <row r="49" ht="36" customHeight="1">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="A49" s="7" t="inlineStr">
         <is>
           <t>TS_TRK_001</t>
         </is>
       </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>TC_TRK_001</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>ALL filter displays complete inventory</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. On /asset-tracking.</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>1. Click 'All Assets' filter tab.</t>
-        </is>
-      </c>
-      <c r="F49" s="5" t="inlineStr">
-        <is>
-          <t>Table shows total inventory matching DB asset count.</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="n"/>
-      <c r="H49" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I49" s="8" t="n"/>
-      <c r="J49" s="5" t="n"/>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>TC_TRK_002</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>AVAILABLE filter shows only available assets</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in.</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Asset Tracking.
+2. Click the "Available Assets" filter tab.
+3. Review all rows.</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>All rows displayed have status AVAILABLE. No assets with other statuses are shown.</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="n"/>
+      <c r="H49" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I49" s="7" t="n"/>
+      <c r="J49" s="6" t="n"/>
     </row>
     <row r="50" ht="36" customHeight="1">
       <c r="A50" s="7" t="inlineStr">
@@ -3120,27 +3294,29 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>TC_TRK_002</t>
+          <t>TC_TRK_003</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>AVAILABLE filter shows only available assets</t>
+          <t>ASSIGNED and OVERDUE filters show correct subsets</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in.</t>
+          <t>Admin is logged in.</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>1. Click 'Available Assets' tab.</t>
+          <t>1. Navigate to Asset Tracking.
+2. Click the "Assigned Assets" tab and review results.
+3. Click the "Overdue Assets" tab and review results.</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>Grid shows only assets with computed status = AVAILABLE.</t>
+          <t>Assigned tab shows only ASSIGNED assets. Overdue tab shows only OVERDUE assets.</t>
         </is>
       </c>
       <c r="G50" s="6" t="n"/>
@@ -3153,44 +3329,46 @@
       <c r="J50" s="6" t="n"/>
     </row>
     <row r="51" ht="36" customHeight="1">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="A51" s="7" t="inlineStr">
         <is>
           <t>TS_TRK_001</t>
         </is>
       </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>TC_TRK_003</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>ASSIGNED and OVERDUE filters show correct subsets</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in.</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>1. Click 'Assigned Assets' tab. 2. Click 'Overdue Assets' tab.</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="inlineStr">
-        <is>
-          <t>Each tab correctly filters to matching computed statuses.</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="n"/>
-      <c r="H51" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I51" s="8" t="n"/>
-      <c r="J51" s="5" t="n"/>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>TC_TRK_004</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>LOST and DAMAGED filters show correct subsets</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in.</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to Asset Tracking.
+2. Click the "Lost Assets" tab and review results.
+3. Click the "Damaged Assets" tab and review results.</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>Lost tab shows only LOST assets. Damaged tab shows DAMAGED or UNDER_REPAIR assets.</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="n"/>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I51" s="7" t="n"/>
+      <c r="J51" s="6" t="n"/>
     </row>
     <row r="52" ht="36" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
@@ -3200,27 +3378,30 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>TC_TRK_004</t>
+          <t>TC_TRK_005</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>LOST and DAMAGED filters show correct subsets</t>
+          <t>Text search filters by Asset Name, Code, and Employee</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in.</t>
+          <t>Admin is logged in. Assets and employee allocations exist.</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>1. Click 'Lost Assets' tab. 2. Click 'Damaged Assets' tab.</t>
+          <t>1. Navigate to Asset Tracking and apply All Assets filter.
+2. Search "AST101" — verify rows are filtered.
+3. Clear and search "Laptop" — verify results.
+4. Clear and search "Carter" — verify results.</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>LOST tab shows status=LOST. DAMAGED tab shows DAMAGED or UNDER_REPAIR assets.</t>
+          <t>Each search term narrows the table to matching rows. Filtered count is less than or equal to the unfiltered total.</t>
         </is>
       </c>
       <c r="G52" s="6" t="n"/>
@@ -3233,44 +3414,46 @@
       <c r="J52" s="6" t="n"/>
     </row>
     <row r="53" ht="36" customHeight="1">
-      <c r="A53" s="8" t="inlineStr">
-        <is>
-          <t>TS_TRK_001</t>
-        </is>
-      </c>
-      <c r="B53" s="8" t="inlineStr">
-        <is>
-          <t>TC_TRK_005</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>Text search filters by Asset Name, Code, and Employee</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in.</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>1. Search 'MacBook'. 2. Search 'AST101'. 3. Search 'Carter'.</t>
-        </is>
-      </c>
-      <c r="F53" s="5" t="inlineStr">
-        <is>
-          <t>Each search narrows rows to matching assets, codes, or employee names respectively.</t>
-        </is>
-      </c>
-      <c r="G53" s="5" t="n"/>
-      <c r="H53" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I53" s="8" t="n"/>
-      <c r="J53" s="5" t="n"/>
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>TS_TCK_001</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>TC_TCK_001</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Raise Ticket form visible only to Employee role</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Admin is logged in.</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>1. Log in as Admin.
+2. Navigate to Ticket Management.
+3. Observe whether the Raise Ticket form is visible.</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>The Raise Ticket form is NOT visible to Admin users. Only employees have access to the ticket creation form.</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="n"/>
+      <c r="H53" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I53" s="7" t="n"/>
+      <c r="J53" s="6" t="n"/>
     </row>
     <row r="54" ht="36" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
@@ -3280,27 +3463,29 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>TC_TCK_001</t>
+          <t>TC_TCK_002</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Raise Ticket form visible only to Employee role</t>
+          <t>Employee can access Ticket Management page after login</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Admin and Employee both logged in.</t>
+          <t>Employee account john.carter@company.com exists.</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>1. Navigate to /ticket-management as Admin. 2. Navigate as Employee.</t>
+          <t>1. Clear session and log in as employee (john.carter@company.com / john123).
+2. Navigate to Ticket Management.
+3. Verify the Raise Ticket form is present.</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>Admin: Raise Ticket form hidden. Employee: form visible.</t>
+          <t>Employee is redirected to /employee-dashboard after login. The Raise Ticket form is visible and accessible on the Ticket Management page.</t>
         </is>
       </c>
       <c r="G54" s="6" t="n"/>
@@ -3313,74 +3498,82 @@
       <c r="J54" s="6" t="n"/>
     </row>
     <row r="55" ht="36" customHeight="1">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="A55" s="7" t="inlineStr">
         <is>
           <t>TS_TCK_001</t>
         </is>
       </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>TC_TCK_002</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>Asset dropdown contains only employee's active assets</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Employee logged in. AST101 assigned, AST102 unassigned.</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>1. Open Asset ID dropdown in Raise Ticket form.</t>
-        </is>
-      </c>
-      <c r="F55" s="5" t="inlineStr">
-        <is>
-          <t>AST101 visible. AST102 excluded.</t>
-        </is>
-      </c>
-      <c r="G55" s="5" t="n"/>
-      <c r="H55" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I55" s="8" t="n"/>
-      <c r="J55" s="5" t="n"/>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>TC_TCK_003</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Employee dashboard is accessible after login</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>Employee account exists. Employee has at least one assigned asset.</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>1. Log in as employee (john.carter@company.com / john123).
+2. Verify redirection to /employee-dashboard.
+3. Navigate to Ticket Management and verify the Raise Ticket form is visible.
+4. Select an active asset, enter a description shorter than 10 characters, and click Create Ticket.</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>Employee dashboard is accessible after login. Raise Ticket form is visible. A validation error is shown for descriptions shorter than 10 characters and no ticket is created.</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="n"/>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="n"/>
+      <c r="J55" s="6" t="n"/>
     </row>
     <row r="56" ht="36" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>TS_TCK_001</t>
+          <t>TS_TCK_002</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>TC_TCK_003</t>
+          <t>TC_TCK_006</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>Description shorter than 10 characters is rejected</t>
+          <t>DAMAGED ticket transitions: PENDING → UNDER_REPAIR → RESOLVED → CLOSED</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Employee logged in.</t>
+          <t>Employee account and admin account exist. Employee has at least one assigned asset.</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>1. Select active asset. 2. Enter 'Broken' (6 chars) as description. 3. Click Create Ticket.</t>
+          <t>1. Log in as employee and raise a DAMAGED ticket.
+2. Log in as Admin and navigate to Ticket Management.
+3. Locate the ticket — verify status is PENDING.
+4. Click "Start Repair" — verify status changes to UNDER_REPAIR.
+5. Click "Resolve" — verify status changes to RESOLVED.
+6. Click "Close" — verify status changes to CLOSED.</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>Validation fails. Message 'Issue description must be at least 10 characters' shown.</t>
+          <t>Ticket transitions through all states: PENDING → UNDER_REPAIR → RESOLVED → CLOSED. Each status change is immediately reflected in the ticket list.</t>
         </is>
       </c>
       <c r="G56" s="6" t="n"/>
@@ -3393,74 +3586,77 @@
       <c r="J56" s="6" t="n"/>
     </row>
     <row r="57" ht="36" customHeight="1">
-      <c r="A57" s="8" t="inlineStr">
-        <is>
-          <t>TS_TCK_001</t>
-        </is>
-      </c>
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>TC_TCK_004</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>Successful ticket creation with DAMAGED issue type</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Employee logged in.</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>1. Select AST101. 2. Issue Type: DAMAGED. 3. Description: 'Screen cracked while traveling'. 4. Click Create Ticket.</t>
-        </is>
-      </c>
-      <c r="F57" s="5" t="inlineStr">
-        <is>
-          <t>Ticket created. Toast '✅ Ticket created successfully' shown. Form resets. Asset status → DAMAGED.</t>
-        </is>
-      </c>
-      <c r="G57" s="5" t="n"/>
-      <c r="H57" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I57" s="8" t="n"/>
-      <c r="J57" s="5" t="n"/>
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>TS_EDH_001</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>TC_EDH_001</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Profile card shows authenticated employee data</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>Employee John Carter (john.carter@company.com) is logged in and on /employee-dashboard.</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>1. Log in as john.carter@company.com.
+2. Navigate to the Employee Dashboard.
+3. Inspect the Profile section.</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>Profile card shows: Employee ID EMP1001, Name "John Carter", Department containing "IT" or "Software", and email john.carter@company.com.</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="n"/>
+      <c r="H57" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I57" s="7" t="n"/>
+      <c r="J57" s="6" t="n"/>
     </row>
     <row r="58" ht="36" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>TS_TCK_001</t>
+          <t>TS_EDH_001</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>TC_TCK_005</t>
+          <t>TC_EDH_002</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>Successful ticket creation with LOST issue type</t>
+          <t>Assigned Assets section shows active allocations</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Employee logged in.</t>
+          <t>Employee is logged in.</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>1. Select AST101. 2. Issue Type: LOST. 3. Description: 'Left headset in office cafeteria'. 4. Click Create Ticket.</t>
+          <t>1. Navigate to the Employee Dashboard.
+2. Locate the Assigned Assets section.</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>Ticket logged. Confirmation message displayed. Ticket appears in employee's ticket table.</t>
+          <t>The Assigned Assets section is visible and shows a non-negative count of assets currently allocated to the employee.</t>
         </is>
       </c>
       <c r="G58" s="6" t="n"/>
@@ -3473,74 +3669,76 @@
       <c r="J58" s="6" t="n"/>
     </row>
     <row r="59" ht="36" customHeight="1">
-      <c r="A59" s="8" t="inlineStr">
-        <is>
-          <t>TS_TCK_002</t>
-        </is>
-      </c>
-      <c r="B59" s="8" t="inlineStr">
-        <is>
-          <t>TC_TCK_006</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>DAMAGED ticket: PENDING → UNDER_REPAIR</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. DAMAGED ticket is PENDING.</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>1. Click 'Start Repair' on ticket. 2. Observe status.</t>
-        </is>
-      </c>
-      <c r="F59" s="5" t="inlineStr">
-        <is>
-          <t>Ticket → UNDER_REPAIR. Asset → UNDER_REPAIR in inventory.</t>
-        </is>
-      </c>
-      <c r="G59" s="5" t="n"/>
-      <c r="H59" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I59" s="8" t="n"/>
-      <c r="J59" s="5" t="n"/>
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>TS_EDH_001</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>TC_EDH_003</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Return History shows completed returns</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>Employee is logged in.</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to the Employee Dashboard.
+2. Locate the Return History section.</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>The Return History section displays a non-negative count of past asset returns.</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="n"/>
+      <c r="H59" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I59" s="7" t="n"/>
+      <c r="J59" s="6" t="n"/>
     </row>
     <row r="60" ht="36" customHeight="1">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>TS_TCK_002</t>
+          <t>TS_EDH_001</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>TC_TCK_007</t>
+          <t>TC_EDH_004</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>DAMAGED ticket: UNDER_REPAIR → RESOLVED</t>
+          <t>Overdue History displays items past deadline</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>Admin logged in. Ticket is UNDER_REPAIR.</t>
+          <t>Employee is logged in.</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>1. Click 'Resolve' on ticket. 2. Observe status.</t>
+          <t>1. Navigate to the Employee Dashboard.
+2. Locate the Overdue History section.</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>Ticket → RESOLVED. Asset → AVAILABLE in inventory.</t>
+          <t>The Overdue History section displays a non-negative count. Overdue items, if any, are listed with relevant details.</t>
         </is>
       </c>
       <c r="G60" s="6" t="n"/>
@@ -3553,322 +3751,127 @@
       <c r="J60" s="6" t="n"/>
     </row>
     <row r="61" ht="36" customHeight="1">
-      <c r="A61" s="8" t="inlineStr">
-        <is>
-          <t>TS_TCK_002</t>
-        </is>
-      </c>
-      <c r="B61" s="8" t="inlineStr">
-        <is>
-          <t>TC_TCK_008</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>DAMAGED ticket: RESOLVED → CLOSED</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. Ticket is RESOLVED.</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>1. Click 'Close' on ticket.</t>
-        </is>
-      </c>
-      <c r="F61" s="5" t="inlineStr">
-        <is>
-          <t>Ticket → CLOSED. Asset remains AVAILABLE.</t>
-        </is>
-      </c>
-      <c r="G61" s="5" t="n"/>
-      <c r="H61" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I61" s="8" t="n"/>
-      <c r="J61" s="5" t="n"/>
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>TS_EDH_001</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>TC_EDH_005</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>Ticket History lists all tickets raised by employee</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>Employee is logged in.</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>1. Navigate to the Employee Dashboard.
+2. Locate the Ticket History section.</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>The Ticket History section displays a non-negative count of tickets raised by the employee.</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="n"/>
+      <c r="H61" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I61" s="7" t="n"/>
+      <c r="J61" s="6" t="n"/>
     </row>
     <row r="62" ht="36" customHeight="1">
-      <c r="A62" s="7" t="inlineStr">
-        <is>
-          <t>TS_TCK_002</t>
-        </is>
-      </c>
-      <c r="B62" s="7" t="inlineStr">
-        <is>
-          <t>TC_TCK_009</t>
-        </is>
-      </c>
-      <c r="C62" s="6" t="inlineStr">
-        <is>
-          <t>LOST ticket: PENDING → UNDER_REVIEW → CLOSED</t>
-        </is>
-      </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>Admin logged in. LOST ticket is PENDING.</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="inlineStr">
-        <is>
-          <t>1. Click 'Under Review'. 2. Then click 'Confirm Lost'.</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="inlineStr">
-        <is>
-          <t>Ticket → CLOSED. Asset → LOST. Employee's assigned list clears. Return history shows LOST.</t>
-        </is>
-      </c>
+      <c r="A62" s="7" t="n"/>
+      <c r="B62" s="7" t="n"/>
+      <c r="C62" s="6" t="n"/>
+      <c r="D62" s="6" t="n"/>
+      <c r="E62" s="6" t="n"/>
+      <c r="F62" s="6" t="n"/>
       <c r="G62" s="6" t="n"/>
-      <c r="H62" s="9" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
+      <c r="H62" s="9" t="n"/>
       <c r="I62" s="7" t="n"/>
       <c r="J62" s="6" t="n"/>
     </row>
     <row r="63" ht="36" customHeight="1">
-      <c r="A63" s="8" t="inlineStr">
-        <is>
-          <t>TS_TCK_002</t>
-        </is>
-      </c>
-      <c r="B63" s="8" t="inlineStr">
-        <is>
-          <t>TC_TCK_010</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>Action buttons change dynamically with ticket status</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Admin logged in. Tickets with statuses PENDING, UNDER_REPAIR, RESOLVED, CLOSED exist.</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>1. Inspect Actions column for each status.</t>
-        </is>
-      </c>
-      <c r="F63" s="5" t="inlineStr">
-        <is>
-          <t>PENDING→Start Repair; UNDER_REPAIR→Resolve; RESOLVED→Close; CLOSED→(no buttons).</t>
-        </is>
-      </c>
-      <c r="G63" s="5" t="n"/>
-      <c r="H63" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I63" s="8" t="n"/>
-      <c r="J63" s="5" t="n"/>
+      <c r="A63" s="7" t="n"/>
+      <c r="B63" s="7" t="n"/>
+      <c r="C63" s="6" t="n"/>
+      <c r="D63" s="6" t="n"/>
+      <c r="E63" s="6" t="n"/>
+      <c r="F63" s="6" t="n"/>
+      <c r="G63" s="6" t="n"/>
+      <c r="H63" s="9" t="n"/>
+      <c r="I63" s="7" t="n"/>
+      <c r="J63" s="6" t="n"/>
     </row>
     <row r="64" ht="36" customHeight="1">
-      <c r="A64" s="7" t="inlineStr">
-        <is>
-          <t>TS_EDH_001</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="inlineStr">
-        <is>
-          <t>TC_EDH_001</t>
-        </is>
-      </c>
-      <c r="C64" s="6" t="inlineStr">
-        <is>
-          <t>Profile card shows authenticated employee data</t>
-        </is>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>Employee logged in (John Carter). On /employee-dashboard.</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
-        <is>
-          <t>1. Inspect 'My Profile' card values.</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>Displays EMP1001, John Carter, IT, john.carter@company.com correctly.</t>
-        </is>
-      </c>
+      <c r="A64" s="7" t="n"/>
+      <c r="B64" s="7" t="n"/>
+      <c r="C64" s="6" t="n"/>
+      <c r="D64" s="6" t="n"/>
+      <c r="E64" s="6" t="n"/>
+      <c r="F64" s="6" t="n"/>
       <c r="G64" s="6" t="n"/>
-      <c r="H64" s="9" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
+      <c r="H64" s="9" t="n"/>
       <c r="I64" s="7" t="n"/>
       <c r="J64" s="6" t="n"/>
     </row>
     <row r="65" ht="36" customHeight="1">
-      <c r="A65" s="8" t="inlineStr">
-        <is>
-          <t>TS_EDH_001</t>
-        </is>
-      </c>
-      <c r="B65" s="8" t="inlineStr">
-        <is>
-          <t>TC_EDH_002</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>Assigned Assets section shows active allocations</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>Employee logged in. Has active allocations.</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>1. View 'Assigned Assets' table. 2. Verify against DB: returned_date IS NULL.</t>
-        </is>
-      </c>
-      <c r="F65" s="5" t="inlineStr">
-        <is>
-          <t>Displays Asset ID, Name, Status, Return Deadline accurately for active records.</t>
-        </is>
-      </c>
-      <c r="G65" s="5" t="n"/>
-      <c r="H65" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I65" s="8" t="n"/>
-      <c r="J65" s="5" t="n"/>
+      <c r="A65" s="7" t="n"/>
+      <c r="B65" s="7" t="n"/>
+      <c r="C65" s="6" t="n"/>
+      <c r="D65" s="6" t="n"/>
+      <c r="E65" s="6" t="n"/>
+      <c r="F65" s="6" t="n"/>
+      <c r="G65" s="6" t="n"/>
+      <c r="H65" s="9" t="n"/>
+      <c r="I65" s="7" t="n"/>
+      <c r="J65" s="6" t="n"/>
     </row>
     <row r="66" ht="36" customHeight="1">
-      <c r="A66" s="7" t="inlineStr">
-        <is>
-          <t>TS_EDH_001</t>
-        </is>
-      </c>
-      <c r="B66" s="7" t="inlineStr">
-        <is>
-          <t>TC_EDH_003</t>
-        </is>
-      </c>
-      <c r="C66" s="6" t="inlineStr">
-        <is>
-          <t>Return History shows completed returns</t>
-        </is>
-      </c>
-      <c r="D66" s="6" t="inlineStr">
-        <is>
-          <t>Employee logged in. Has past returned assets.</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="inlineStr">
-        <is>
-          <t>1. View 'Return History' table.</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="inlineStr">
-        <is>
-          <t>Displays asset name, return date, status (RETURNED or LOST), and remarks.</t>
-        </is>
-      </c>
+      <c r="A66" s="7" t="n"/>
+      <c r="B66" s="7" t="n"/>
+      <c r="C66" s="6" t="n"/>
+      <c r="D66" s="6" t="n"/>
+      <c r="E66" s="6" t="n"/>
+      <c r="F66" s="6" t="n"/>
       <c r="G66" s="6" t="n"/>
-      <c r="H66" s="9" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
+      <c r="H66" s="9" t="n"/>
       <c r="I66" s="7" t="n"/>
       <c r="J66" s="6" t="n"/>
     </row>
     <row r="67" ht="36" customHeight="1">
-      <c r="A67" s="8" t="inlineStr">
-        <is>
-          <t>TS_EDH_001</t>
-        </is>
-      </c>
-      <c r="B67" s="8" t="inlineStr">
-        <is>
-          <t>TC_EDH_004</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>Overdue History displays items past deadline</t>
-        </is>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>Employee logged in. Has an allocation with deadline &lt; today and no return.</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>1. View 'Overdue History' table.</t>
-        </is>
-      </c>
-      <c r="F67" s="5" t="inlineStr">
-        <is>
-          <t>Asset name, deadline, and red OVERDUE badge are shown.</t>
-        </is>
-      </c>
-      <c r="G67" s="5" t="n"/>
-      <c r="H67" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I67" s="8" t="n"/>
-      <c r="J67" s="5" t="n"/>
+      <c r="A67" s="7" t="n"/>
+      <c r="B67" s="7" t="n"/>
+      <c r="C67" s="6" t="n"/>
+      <c r="D67" s="6" t="n"/>
+      <c r="E67" s="6" t="n"/>
+      <c r="F67" s="6" t="n"/>
+      <c r="G67" s="6" t="n"/>
+      <c r="H67" s="9" t="n"/>
+      <c r="I67" s="7" t="n"/>
+      <c r="J67" s="6" t="n"/>
     </row>
     <row r="68" ht="36" customHeight="1">
-      <c r="A68" s="7" t="inlineStr">
-        <is>
-          <t>TS_EDH_001</t>
-        </is>
-      </c>
-      <c r="B68" s="7" t="inlineStr">
-        <is>
-          <t>TC_EDH_005</t>
-        </is>
-      </c>
-      <c r="C68" s="6" t="inlineStr">
-        <is>
-          <t>Ticket History lists all tickets raised by employee</t>
-        </is>
-      </c>
-      <c r="D68" s="6" t="inlineStr">
-        <is>
-          <t>Employee logged in. Has raised tickets.</t>
-        </is>
-      </c>
-      <c r="E68" s="6" t="inlineStr">
-        <is>
-          <t>1. View 'Ticket History' table.</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="inlineStr">
-        <is>
-          <t>Lists asset name, issue description, and current ticket status (e.g. CLOSED).</t>
-        </is>
-      </c>
+      <c r="A68" s="7" t="n"/>
+      <c r="B68" s="7" t="n"/>
+      <c r="C68" s="6" t="n"/>
+      <c r="D68" s="6" t="n"/>
+      <c r="E68" s="6" t="n"/>
+      <c r="F68" s="6" t="n"/>
       <c r="G68" s="6" t="n"/>
-      <c r="H68" s="9" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
+      <c r="H68" s="9" t="n"/>
       <c r="I68" s="7" t="n"/>
       <c r="J68" s="6" t="n"/>
     </row>
@@ -3886,7 +3889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3907,15 +3910,15 @@
           <t>CAMS – Defect Tracking Log</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
+      <c r="F1" s="11" t="n"/>
+      <c r="G1" s="11" t="n"/>
+      <c r="H1" s="11" t="n"/>
+      <c r="I1" s="11" t="n"/>
+      <c r="J1" s="12" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="n"/>
@@ -4034,52 +4037,52 @@
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>DF_002</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Delete employee confirmation dialog not always triggered</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Employee Management</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>1. Go to Employee Management. 2. Click Delete on any employee.</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Browser confirmation prompt must appear before deletion.</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Request sent immediately without confirmation dialog in some cases.</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>Developer UI Team</t>
         </is>
@@ -4138,52 +4141,52 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>DF_004</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Asset assignment allows past return deadline</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Asset Assignment</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>1. Fill assignment form. 2. Set Return Deadline to yesterday. 3. Click Assign Asset.</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>System blocks submission: 'Return Deadline cannot be in the past'.</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Assignment succeeds; record created with immediate OVERDUE status.</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>API Gateway Team</t>
         </is>
@@ -4240,6 +4243,42 @@
           <t>Frontend Dev Team</t>
         </is>
       </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="7" t="n"/>
+      <c r="J10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="7" t="n"/>
+      <c r="J11" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>